<commit_message>
Final adjustments to notebook 2
</commit_message>
<xml_diff>
--- a/scripts/eeg/subjects_processing_stage.xlsx
+++ b/scripts/eeg/subjects_processing_stage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahm\projects\loc_analysis\scripts\eeg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD579A5-9A2E-47EA-8225-13E1F5897BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35183516-4460-4F25-80B9-6B21281410E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="12">
   <si>
     <t>sub</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>note</t>
-  </si>
-  <si>
-    <t>2: manual config</t>
   </si>
   <si>
     <t>process</t>
@@ -314,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -342,7 +339,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -360,131 +356,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -507,11 +386,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -529,63 +408,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1494,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D82AE40D-4653-447C-9679-4F72663E49E3}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
@@ -1504,54 +1327,49 @@
     <col min="8" max="8" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="16" t="s">
+    <row r="1" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="16" t="s">
+      <c r="D2" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="16" t="s">
+      <c r="F2" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="21"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="21"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="12">
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="11">
         <v>3</v>
       </c>
-      <c r="C3" s="13">
-        <v>0</v>
-      </c>
-      <c r="D3" s="13">
-        <v>1</v>
-      </c>
-      <c r="E3" s="19"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="12">
+        <v>0</v>
+      </c>
+      <c r="D3" s="12">
+        <v>1</v>
+      </c>
+      <c r="E3" s="18"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="6">
         <v>4</v>
       </c>
@@ -1561,17 +1379,14 @@
       <c r="D4" s="5">
         <v>1</v>
       </c>
-      <c r="E4" s="20"/>
+      <c r="E4" s="19"/>
       <c r="F4" s="5"/>
-      <c r="G4" s="13"/>
+      <c r="G4" s="12"/>
       <c r="H4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-    </row>
-    <row r="5" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="5" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="6">
         <v>9</v>
       </c>
@@ -1581,17 +1396,14 @@
       <c r="D5" s="5">
         <v>1</v>
       </c>
-      <c r="E5" s="20"/>
+      <c r="E5" s="19"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="13"/>
+      <c r="G5" s="12"/>
       <c r="H5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-    </row>
-    <row r="6" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="6" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B6" s="6">
         <v>10</v>
       </c>
@@ -1601,17 +1413,14 @@
       <c r="D6" s="5">
         <v>1</v>
       </c>
-      <c r="E6" s="20"/>
+      <c r="E6" s="19"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="13"/>
+      <c r="G6" s="12"/>
       <c r="H6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-    </row>
-    <row r="7" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="6">
         <v>11</v>
       </c>
@@ -1621,14 +1430,14 @@
       <c r="D7" s="5">
         <v>1</v>
       </c>
-      <c r="E7" s="20"/>
+      <c r="E7" s="19"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="13"/>
+      <c r="G7" s="12"/>
       <c r="H7" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="6">
         <v>12</v>
       </c>
@@ -1638,14 +1447,14 @@
       <c r="D8" s="5">
         <v>1</v>
       </c>
-      <c r="E8" s="20"/>
+      <c r="E8" s="19"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="13"/>
+      <c r="G8" s="12"/>
       <c r="H8" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="6">
         <v>17</v>
       </c>
@@ -1659,13 +1468,12 @@
         <v>0</v>
       </c>
       <c r="F9" s="5"/>
-      <c r="G9" s="13"/>
+      <c r="G9" s="12"/>
       <c r="H9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="L9" s="21"/>
-    </row>
-    <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="6">
         <v>20</v>
       </c>
@@ -1679,16 +1487,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>12</v>
-      </c>
       <c r="H10" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="6">
         <v>21</v>
       </c>
@@ -1702,12 +1510,12 @@
         <v>0</v>
       </c>
       <c r="F11" s="5"/>
-      <c r="G11" s="13"/>
+      <c r="G11" s="12"/>
       <c r="H11" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="6">
         <v>22</v>
       </c>
@@ -1721,12 +1529,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="5"/>
-      <c r="G12" s="13"/>
+      <c r="G12" s="12"/>
       <c r="H12" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="6">
         <v>23</v>
       </c>
@@ -1740,12 +1548,12 @@
         <v>0</v>
       </c>
       <c r="F13" s="5"/>
-      <c r="G13" s="13"/>
+      <c r="G13" s="12"/>
       <c r="H13" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="6">
         <v>26</v>
       </c>
@@ -1757,12 +1565,12 @@
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-      <c r="G14" s="13"/>
+      <c r="G14" s="12"/>
       <c r="H14" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B15" s="6">
         <v>27</v>
       </c>
@@ -1774,12 +1582,12 @@
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
-      <c r="G15" s="13"/>
+      <c r="G15" s="12"/>
       <c r="H15" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B16" s="6">
         <v>29</v>
       </c>
@@ -1791,7 +1599,7 @@
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="13"/>
+      <c r="G16" s="12"/>
       <c r="H16" s="7" t="s">
         <v>7</v>
       </c>
@@ -1808,7 +1616,7 @@
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="13"/>
+      <c r="G17" s="12"/>
       <c r="H17" s="7" t="s">
         <v>7</v>
       </c>
@@ -1825,7 +1633,7 @@
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="13"/>
+      <c r="G18" s="12"/>
       <c r="H18" s="7" t="s">
         <v>7</v>
       </c>
@@ -1842,7 +1650,7 @@
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="13"/>
+      <c r="G19" s="12"/>
       <c r="H19" s="7" t="s">
         <v>7</v>
       </c>
@@ -1859,7 +1667,7 @@
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="13"/>
+      <c r="G20" s="12"/>
       <c r="H20" s="7" t="s">
         <v>7</v>
       </c>
@@ -1876,7 +1684,7 @@
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
-      <c r="G21" s="13"/>
+      <c r="G21" s="12"/>
       <c r="H21" s="7" t="s">
         <v>7</v>
       </c>
@@ -1893,7 +1701,7 @@
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
-      <c r="G22" s="13"/>
+      <c r="G22" s="12"/>
       <c r="H22" s="7" t="s">
         <v>7</v>
       </c>
@@ -1910,7 +1718,7 @@
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
-      <c r="G23" s="13"/>
+      <c r="G23" s="12"/>
       <c r="H23" s="7" t="s">
         <v>7</v>
       </c>
@@ -1927,7 +1735,7 @@
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="13"/>
+      <c r="G24" s="12"/>
       <c r="H24" s="7" t="s">
         <v>7</v>
       </c>
@@ -1944,7 +1752,7 @@
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
-      <c r="G25" s="13"/>
+      <c r="G25" s="12"/>
       <c r="H25" s="7" t="s">
         <v>7</v>
       </c>
@@ -1961,7 +1769,7 @@
       </c>
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
-      <c r="G26" s="13"/>
+      <c r="G26" s="12"/>
       <c r="H26" s="7" t="s">
         <v>7</v>
       </c>
@@ -1980,25 +1788,25 @@
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="16" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E27">
-    <cfRule type="expression" dxfId="8" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula xml:space="preserve"> $D3 = 1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H27">
-    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="1: BIDS">
-      <formula>NOT(ISERROR(SEARCH("1: BIDS",H3)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="3: preprocessed">
+      <formula>NOT(ISERROR(SEARCH("3: preprocessed",H3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="5" operator="containsText" text="2: manual config">
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="2: manual config">
       <formula>NOT(ISERROR(SEARCH("2: manual config",H3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="3: preprocessed">
-      <formula>NOT(ISERROR(SEARCH("3: preprocessed",H3)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="1: BIDS">
+      <formula>NOT(ISERROR(SEARCH("1: BIDS",H3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>

<commit_message>
More detailed commentation for notebook 3
</commit_message>
<xml_diff>
--- a/scripts/eeg/subjects_processing_stage.xlsx
+++ b/scripts/eeg/subjects_processing_stage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahm\projects\loc_analysis\scripts\eeg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85212E82-80D8-4E6E-9A26-DC5E5EF3CE3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B137AD0D-988D-4F21-96DA-4BB5493B5E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="18">
   <si>
     <t>sub</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t>enc_start and first few trials were not recorded</t>
+  </si>
+  <si>
+    <t>Many frontal channels are noisy</t>
   </si>
 </sst>
 </file>
@@ -1716,11 +1719,15 @@
       <c r="D20" s="5">
         <v>0</v>
       </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G20" s="12"/>
       <c r="H20" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1733,11 +1740,15 @@
       <c r="D21" s="5">
         <v>0</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G21" s="12"/>
       <c r="H21" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1750,11 +1761,15 @@
       <c r="D22" s="5">
         <v>0</v>
       </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G22" s="12"/>
       <c r="H22" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1767,11 +1782,15 @@
       <c r="D23" s="5">
         <v>0</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G23" s="12"/>
       <c r="H23" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1784,11 +1803,15 @@
       <c r="D24" s="4">
         <v>0</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+      <c r="E24" s="4">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G24" s="12"/>
       <c r="H24" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1801,11 +1824,15 @@
       <c r="D25" s="5">
         <v>0</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="E25" s="5">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G25" s="12"/>
       <c r="H25" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1818,11 +1845,17 @@
       <c r="D26" s="5">
         <v>0</v>
       </c>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="12"/>
+      <c r="E26" s="5">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="H26" s="7" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1836,11 +1869,17 @@
       <c r="D27" s="10">
         <v>0</v>
       </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="E27" s="10">
+        <v>0</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>17</v>
+      </c>
       <c r="H27" s="16" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalized first QC section of Notebook 4, 2.1
</commit_message>
<xml_diff>
--- a/scripts/eeg/subjects_processing_stage.xlsx
+++ b/scripts/eeg/subjects_processing_stage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahm\projects\loc_analysis\scripts\eeg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DF0771-6D41-4070-BB8D-638EB37B366F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3E72B1-B07C-4376-927F-42DB1C6A4EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-27090" yWindow="1815" windowWidth="14400" windowHeight="7275" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="eeg_analysis" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="15">
   <si>
     <t>sub</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Many frontal channels are noisy</t>
   </si>
   <si>
-    <t>Laura/Javier: Adjust data curation?</t>
-  </si>
-  <si>
     <t>enc_start and first trials were not recorded</t>
   </si>
   <si>
@@ -88,10 +85,7 @@
     <t>Subjects preprocessed:</t>
   </si>
   <si>
-    <t>Laura/Javier: Adjust data curation? Enc. Trial 13 missing</t>
-  </si>
-  <si>
-    <t>Laura/Javier: Adjust data curation? Enc. Trial 64 missing</t>
+    <t>BLOCKER: fix bug in behavioral data (missing enc trial)</t>
   </si>
 </sst>
 </file>
@@ -437,22 +431,7 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp"/>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -481,6 +460,11 @@
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp"/>
       </fill>
     </dxf>
   </dxfs>
@@ -780,7 +764,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -832,7 +816,7 @@
       </c>
       <c r="G6" s="13"/>
       <c r="I6" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J6" s="20">
         <f>COUNTA(B5:B46)</f>
@@ -853,7 +837,7 @@
       </c>
       <c r="G7" s="13"/>
       <c r="I7" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J7" s="21">
         <f>COUNTIF(C:C, 0)</f>
@@ -874,7 +858,7 @@
       </c>
       <c r="G8" s="13"/>
       <c r="I8" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J8" s="22">
         <f>COUNTIF(F:F,"3: preprocessed")</f>
@@ -1078,7 +1062,7 @@
         <v>5</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1096,7 +1080,7 @@
         <v>5</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1114,7 +1098,7 @@
         <v>5</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1132,7 +1116,7 @@
         <v>5</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1150,7 +1134,7 @@
         <v>5</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1168,7 +1152,7 @@
         <v>5</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1188,7 +1172,7 @@
         <v>5</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1526,20 +1510,20 @@
       <sortCondition ref="F4"/>
     </sortState>
   </autoFilter>
+  <conditionalFormatting sqref="B5:G46">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$C5 = 1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F5:F46 I6:I8">
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="3: preprocessed">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="3: preprocessed">
       <formula>NOT(ISERROR(SEARCH("3: preprocessed",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="2: manual config">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="2: manual config">
       <formula>NOT(ISERROR(SEARCH("2: manual config",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="1: BIDS">
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="1: BIDS">
       <formula>NOT(ISERROR(SEARCH("1: BIDS",F5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:G46">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$C5 = 1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>